<commit_message>
Just saving the means for some plots
</commit_message>
<xml_diff>
--- a/Cell survival results/PM_means.xlsx
+++ b/Cell survival results/PM_means.xlsx
@@ -425,256 +425,369 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dose</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Dose</t>
+          <t>Mean Survival</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Mean Survival</t>
+          <t>STD</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>STD</t>
+          <t>Experiment</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Experiment</t>
+          <t>c</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1260936497896067</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EXP_2026_2_26</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>#008080</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.3618403805853483</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.04422081792636776</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EXP_2026_2_26</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>#008080</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.05363352717533893</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.005191153366031996</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EXP_2026_2_26</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>#008080</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.001759189357321175</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0007288743821023127</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EXP_2026_2_26</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>#008080</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+      <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="n">
-        <v>0.1260936497896067</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>EXP_2026_2_26</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="C6" t="n">
+        <v>0.1053728227082863</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_02</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>#FF00FF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.1913833095775407</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.06149536973037455</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_02</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>#FF00FF</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.02318105013203637</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.004092318237677244</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_02</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>#FF00FF</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.001033107478647169</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5.848880936810855e-05</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_02</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>#FF00FF</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
         <v>0</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.222952782016584</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_18</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
-        <v>0.3618403805853483</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.04422081792636776</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>EXP_2026_2_26</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="B11" t="n">
+        <v>0.06493514499426514</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.04277493394358996</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_18</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.008583959522924048</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0008772552339908354</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_18</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.001206150580748194</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0005688287184585851</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_18</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>#008000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
         <v>0</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.1013460046033881</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_19</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>#00FF00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.3067661509841179</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.01453829043062222</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_19</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>#00FF00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
         <v>5</v>
       </c>
-      <c r="C4" t="n">
-        <v>0.05363352717533893</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.005191153366031996</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>EXP_2026_2_26</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B5" t="n">
+      <c r="B16" t="n">
+        <v>0.01784439404550058</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.001737452301901615</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>EXP_2026_3_19</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>#00FF00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
         <v>8</v>
       </c>
-      <c r="C5" t="n">
-        <v>0.001759189357321175</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.0007288743821023127</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>EXP_2026_2_26</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.1013460046033881</v>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="B17" t="n">
+        <v>0.0009549433341824351</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.000187685361286627</v>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>EXP_2026_3_19</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.3067661509841179</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.01453829043062222</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_19</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.01784439404550058</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.001737452301901615</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_19</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B9" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.0009549433341824351</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.000187685361286627</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_19</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.1053728227082863</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.1913833095775407</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.06149536973037455</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B12" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.02318105013203637</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.004092318237677244</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B13" t="n">
-        <v>8</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.001033107478647169</v>
-      </c>
-      <c r="D13" t="n">
-        <v>5.848880936810855e-05</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>EXP_2026_3_2</t>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>#00FF00</t>
         </is>
       </c>
     </row>

</xml_diff>